<commit_message>
Fixed border in .xlsx template
</commit_message>
<xml_diff>
--- a/api/templates/error_rate/en.xlsx
+++ b/api/templates/error_rate/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26026"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\error_rate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\error_rate\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED591FC5-A6D2-42D3-BBF2-3B3F6E1EDA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2004" yWindow="1524" windowWidth="20568" windowHeight="10836" tabRatio="815"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="6" r:id="rId1"/>
@@ -18,15 +19,6 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -136,7 +128,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
@@ -215,72 +207,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -308,40 +240,74 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -391,49 +357,41 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="4" xfId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="4" xfId="43" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -506,7 +464,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -843,14 +801,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="27.09765625" customWidth="1"/>
     <col min="3" max="3" width="16.3984375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="27.09765625" customWidth="1"/>
-    <col min="6" max="6" width="16.8984375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="16.8984375" style="4" customWidth="1"/>
     <col min="7" max="7" width="14.8984375" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
   </cols>
@@ -884,75 +842,68 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+    <row r="8" spans="1:9" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F8" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G8" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H8" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I8" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I9" s="11" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -961,8 +912,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.8984375" customWidth="1"/>
@@ -971,7 +922,7 @@
     <col min="4" max="4" width="33.8984375" customWidth="1"/>
     <col min="5" max="5" width="20.59765625" customWidth="1"/>
     <col min="6" max="6" width="19.59765625" customWidth="1"/>
-    <col min="7" max="7" width="16.59765625" style="11" customWidth="1"/>
+    <col min="7" max="7" width="16.59765625" style="4" customWidth="1"/>
     <col min="8" max="8" width="14.8984375" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
@@ -1006,90 +957,82 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="7" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+    <row r="8" spans="1:10" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G8" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H8" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I8" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J8" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="J9" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1103,12 +1046,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.09765625" customWidth="1"/>
-    <col min="2" max="2" width="16.5" style="11" customWidth="1"/>
+    <col min="2" max="2" width="16.5" style="4" customWidth="1"/>
     <col min="3" max="3" width="14.8984375" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
@@ -1123,50 +1066,47 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="4" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    <row r="5" spans="1:5" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D5" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E5" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E6" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Showing in reports only the devices that perform results
</commit_message>
<xml_diff>
--- a/api/templates/error_rate/en.xlsx
+++ b/api/templates/error_rate/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26130"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\error_rate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\error_rate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED591FC5-A6D2-42D3-BBF2-3B3F6E1EDA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3070E171-44CE-4D3B-BD8A-4E63666553D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="6" r:id="rId1"/>
@@ -35,9 +35,6 @@
     <t>Date Range: &lt;Dates&gt;</t>
   </si>
   <si>
-    <t>Last Upload</t>
-  </si>
-  <si>
     <t>Error Rate</t>
   </si>
   <si>
@@ -123,6 +120,9 @@
   </si>
   <si>
     <t>&lt;senderOperator&gt;</t>
+  </si>
+  <si>
+    <t>Last Result Update</t>
   </si>
 </sst>
 </file>
@@ -815,7 +815,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -829,80 +829,80 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>10</v>
-      </c>
       <c r="F8" s="13" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>0</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>21</v>
-      </c>
       <c r="I9" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -929,7 +929,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -944,86 +944,86 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>6</v>
-      </c>
       <c r="C8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="E8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>10</v>
-      </c>
       <c r="G8" s="13" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" s="14" t="s">
         <v>0</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>30</v>
-      </c>
       <c r="C9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="I9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>21</v>
-      </c>
       <c r="J9" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -1058,7 +1058,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1068,41 +1068,41 @@
     </row>
     <row r="4" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="12" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>21</v>
-      </c>
       <c r="E6" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>